<commit_message>
Implementados testes de estoque, patrimônio e depreciação.
</commit_message>
<xml_diff>
--- a/manual_values/202605.xlsx
+++ b/manual_values/202605.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\contabilidade\PhpstormProjects\tester\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\contabilidade\PhpstormProjects\tester\manual_values\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC3166D7-93D8-4B36-B823-389B3E86E3A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ECE672B-62A4-4311-A9A2-E998560571B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1A150101-511F-452C-8ABB-F5FAD95197D8}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1A150101-511F-452C-8ABB-F5FAD95197D8}"/>
   </bookViews>
   <sheets>
     <sheet name="PM" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="64">
   <si>
     <t>Ativo - saldo inicial</t>
   </si>
@@ -225,6 +225,15 @@
   </si>
   <si>
     <t>valor</t>
+  </si>
+  <si>
+    <t>Estoque - saldo final</t>
+  </si>
+  <si>
+    <t>Patrimônio - saldo final</t>
+  </si>
+  <si>
+    <t>Depreciação - débito</t>
   </si>
 </sst>
 </file>
@@ -382,30 +391,30 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5B1B4944-F349-46BE-8828-FA50192B85E7}" name="VALORES_MANUAIS" displayName="VALORES_MANUAIS" ref="A1:B60" totalsRowShown="0" headerRowDxfId="7">
-  <autoFilter ref="A1:B60" xr:uid="{E45FC8DF-0BB6-4032-80FB-F4013350F743}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5B1B4944-F349-46BE-8828-FA50192B85E7}" name="VALORES_MANUAIS" displayName="VALORES_MANUAIS" ref="A1:B63" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:B63" xr:uid="{E45FC8DF-0BB6-4032-80FB-F4013350F743}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{72E397A3-A743-4EEA-BFD5-3113ADB13208}" name="item"/>
-    <tableColumn id="2" xr3:uid="{67920E14-6B74-4A39-9EF1-9C6C10986B72}" name="valor" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{67920E14-6B74-4A39-9EF1-9C6C10986B72}" name="valor" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FF865E16-590A-4D5C-AA1B-EFB77009CF30}" name="VALORES_MANUAIS3" displayName="VALORES_MANUAIS3" ref="A1:B60" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:B60" xr:uid="{E45FC8DF-0BB6-4032-80FB-F4013350F743}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FF865E16-590A-4D5C-AA1B-EFB77009CF30}" name="VALORES_MANUAIS3" displayName="VALORES_MANUAIS3" ref="A1:B63" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:B63" xr:uid="{E45FC8DF-0BB6-4032-80FB-F4013350F743}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{C1C2EB70-F2D2-444D-865E-280D38957574}" name="item"/>
-    <tableColumn id="3" xr3:uid="{842F6FAD-82EB-4A9E-86D9-2A2DE6AF4FD5}" name="valor" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{842F6FAD-82EB-4A9E-86D9-2A2DE6AF4FD5}" name="valor" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{37ED8C2D-15EB-4F6E-A638-6BC4E60C9654}" name="VALORES_MANUAIS34" displayName="VALORES_MANUAIS34" ref="A1:B60" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:B60" xr:uid="{E45FC8DF-0BB6-4032-80FB-F4013350F743}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{37ED8C2D-15EB-4F6E-A638-6BC4E60C9654}" name="VALORES_MANUAIS34" displayName="VALORES_MANUAIS34" ref="A1:B63" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:B63" xr:uid="{E45FC8DF-0BB6-4032-80FB-F4013350F743}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{BD7E1018-7838-45B2-82AE-AE2BEDD67274}" name="item"/>
     <tableColumn id="4" xr3:uid="{0A114F86-24FC-45B6-B43E-98F351D49B74}" name="valor" dataDxfId="2"/>
@@ -415,8 +424,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FEED078D-EBA6-4FAB-BCB9-9C62671019E4}" name="VALORES_MANUAIS345" displayName="VALORES_MANUAIS345" ref="A1:B60" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:B60" xr:uid="{E45FC8DF-0BB6-4032-80FB-F4013350F743}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FEED078D-EBA6-4FAB-BCB9-9C62671019E4}" name="VALORES_MANUAIS345" displayName="VALORES_MANUAIS345" ref="A1:B63" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:B63" xr:uid="{E45FC8DF-0BB6-4032-80FB-F4013350F743}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{B4A09C18-EEA3-4FF9-85C2-5502AE150477}" name="item"/>
     <tableColumn id="5" xr3:uid="{01FDB2A1-F6A9-4341-A31E-CC051538A3C2}" name="valor" dataDxfId="0">
@@ -747,7 +756,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.140625" bestFit="1" customWidth="1"/>
@@ -1232,6 +1241,30 @@
       </c>
       <c r="B60" s="2">
         <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>61</v>
+      </c>
+      <c r="B61" s="2">
+        <v>833786.93</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62" s="2">
+        <v>18107149.149999999</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B63" s="2">
+        <v>110911.37</v>
       </c>
     </row>
   </sheetData>
@@ -1247,7 +1280,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.140625" bestFit="1" customWidth="1"/>
@@ -1726,6 +1759,30 @@
       </c>
       <c r="B60" s="2">
         <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>61</v>
+      </c>
+      <c r="B61" s="2">
+        <v>3528.9700000000003</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62" s="2">
+        <v>94205.14</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B63" s="2">
+        <v>1048.3</v>
       </c>
     </row>
   </sheetData>
@@ -1741,7 +1798,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.140625" bestFit="1" customWidth="1"/>
@@ -2227,6 +2284,24 @@
       <c r="B60" s="2">
         <v>0</v>
       </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>61</v>
+      </c>
+      <c r="B61" s="3"/>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62" s="3"/>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B63" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -2241,7 +2316,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.140625" bestFit="1" customWidth="1"/>
@@ -2787,6 +2862,33 @@
         <v>0</v>
       </c>
     </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>61</v>
+      </c>
+      <c r="B61" s="2">
+        <f>SUM(_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS[item],VALORES_MANUAIS[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS3[item],VALORES_MANUAIS3[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS34[item],VALORES_MANUAIS34[valor],0))</f>
+        <v>837315.9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62" s="2">
+        <f>SUM(_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS[item],VALORES_MANUAIS[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS3[item],VALORES_MANUAIS3[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS34[item],VALORES_MANUAIS34[valor],0))</f>
+        <v>18201354.289999999</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B63" s="2">
+        <f>SUM(_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS[item],VALORES_MANUAIS[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS3[item],VALORES_MANUAIS3[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS34[item],VALORES_MANUAIS34[valor],0))</f>
+        <v>111959.67</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Alterada rotina para seleção de testes. Agora não considera o sufixo -test.php, apenas .php
Isso evita que algum teste não seja executado por não ter o sufixo -test no nome.
</commit_message>
<xml_diff>
--- a/manual_values/202605.xlsx
+++ b/manual_values/202605.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\contabilidade\PhpstormProjects\tester\manual_values\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ECE672B-62A4-4311-A9A2-E998560571B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674B21FE-6877-4F2F-AF9C-C4276F02F62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1A150101-511F-452C-8ABB-F5FAD95197D8}"/>
+    <workbookView xWindow="22395" yWindow="0" windowWidth="6510" windowHeight="15585" xr2:uid="{1A150101-511F-452C-8ABB-F5FAD95197D8}"/>
   </bookViews>
   <sheets>
     <sheet name="PM" sheetId="1" r:id="rId1"/>
@@ -976,7 +976,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>60730861.810000002</v>
+        <v>60745022.82</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -992,7 +992,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>126298251.44</v>
+        <v>126312412.45</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -1016,7 +1016,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>161376898.46000001</v>
+        <v>161391059.47</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -1024,7 +1024,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>126298251.44</v>
+        <v>126312412.45</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="B27" s="2">
         <f>SUM(_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS[item],VALORES_MANUAIS[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS3[item],VALORES_MANUAIS3[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS34[item],VALORES_MANUAIS34[valor],0))</f>
-        <v>66694186.300000004</v>
+        <v>66708347.310000002</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -2580,7 +2580,7 @@
       </c>
       <c r="B29" s="2">
         <f>SUM(_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS[item],VALORES_MANUAIS[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS3[item],VALORES_MANUAIS3[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS34[item],VALORES_MANUAIS34[valor],0))</f>
-        <v>179650637.09999999</v>
+        <v>179664798.11000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="B32" s="2">
         <f>SUM(_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS[item],VALORES_MANUAIS[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS3[item],VALORES_MANUAIS3[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS34[item],VALORES_MANUAIS34[valor],0))</f>
-        <v>184182625.43000001</v>
+        <v>184196786.44</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="B33" s="2">
         <f>SUM(_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS[item],VALORES_MANUAIS[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS3[item],VALORES_MANUAIS3[valor],0),_xlfn.XLOOKUP(VALORES_MANUAIS345[[#This Row],[item]],VALORES_MANUAIS34[item],VALORES_MANUAIS34[valor],0))</f>
-        <v>179650637.09999999</v>
+        <v>179664798.11000001</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>